<commit_message>
Finalisation des fonctionnalités administrateur
</commit_message>
<xml_diff>
--- a/InfosUtilisateursSite.xlsx
+++ b/InfosUtilisateursSite.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemai\Documents\13_ProjetsPro\1_FormationDevWeb_2022_2023\Site_E-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A375F4-9DCE-401C-8720-8167A1F512CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B42332-36CB-4CC8-8916-E312DE116501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5565" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="63">
   <si>
     <t>Nom</t>
   </si>
@@ -208,13 +208,21 @@
   </si>
   <si>
     <t>Tlemaire03022002.</t>
+  </si>
+  <si>
+    <t>USER temporaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A rajouter
+Apres
+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,13 +238,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -266,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -276,6 +296,33 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -560,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D2:L12"/>
+  <dimension ref="D2:M12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="12.90625" customWidth="1"/>
@@ -570,9 +617,10 @@
     <col min="9" max="9" width="12.08984375" customWidth="1"/>
     <col min="10" max="10" width="12.54296875" customWidth="1"/>
     <col min="11" max="11" width="16.7265625" customWidth="1"/>
+    <col min="13" max="13" width="16.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:12" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="4:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D2" s="1" t="s">
         <v>59</v>
       </c>
@@ -601,7 +649,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="4:12" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="4:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D3" s="4">
         <v>70</v>
       </c>
@@ -630,7 +678,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="4:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="4:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D4" s="4">
         <v>71</v>
       </c>
@@ -659,7 +707,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="4:12" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="4:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D5" s="4">
         <v>72</v>
       </c>
@@ -688,7 +736,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="4:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="4:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D6" s="4">
         <v>73</v>
       </c>
@@ -717,7 +765,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="4:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D7" s="4">
         <v>74</v>
       </c>
@@ -745,153 +793,166 @@
       <c r="L7" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="4:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D8" s="4">
+      <c r="M7" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="4:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="8">
         <v>75</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="9">
         <v>667890123</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="10">
         <v>36783</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" spans="4:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D9" s="4">
+      <c r="M8" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D9" s="8">
         <v>76</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="9">
         <v>678901234</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="10">
         <v>34670</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="4:12" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="4">
+      <c r="M9" s="13"/>
+    </row>
+    <row r="10" spans="4:13" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="8">
         <v>77</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="9">
         <v>689012345</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="10">
         <v>35541</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="4:12" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D11" s="4">
+      <c r="M10" s="13"/>
+    </row>
+    <row r="11" spans="4:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="8">
         <v>78</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="9">
         <v>690123456</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="10">
         <v>33460</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D12" s="4">
+      <c r="M11" s="13"/>
+    </row>
+    <row r="12" spans="4:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="5">
         <v>79</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="6">
         <v>601234567</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="7">
         <v>36285</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" s="6" t="s">
         <v>38</v>
       </c>
+      <c r="M12" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="M8:M12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
debut de la refonte de la page d accueil, ajout de plusieurs commentaires pour eviter les bug visuel de l IDE, l utilisateur peut maintenant supprimer son compte, le bouton annuler dans la page de modif mot de passe est corriger, il renvoie maintenant dans le compte utilisateur
</commit_message>
<xml_diff>
--- a/InfosUtilisateursSite.xlsx
+++ b/InfosUtilisateursSite.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemai\Documents\13_ProjetsPro\1_FormationDevWeb_2022_2023\Site_E-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B42332-36CB-4CC8-8916-E312DE116501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B279E1FE-7C08-4B5B-824A-E84CBE95C6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5565" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -210,7 +210,7 @@
     <t>Tlemaire03022002.</t>
   </si>
   <si>
-    <t>USER temporaire</t>
+    <t>USER Temporaire</t>
   </si>
   <si>
     <t xml:space="preserve">A rajouter
@@ -259,7 +259,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -282,11 +282,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -321,11 +358,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -706,96 +746,101 @@
       <c r="L4" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="M4" s="11" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="5" spans="4:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="4">
+      <c r="D5" s="8">
         <v>72</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="9">
         <v>634567890</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="10">
         <v>36107</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="9" t="s">
         <v>13</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D6" s="4">
+      <c r="D6" s="8">
         <v>73</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="9">
         <v>645678901</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="10">
         <v>32892</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="9" t="s">
         <v>13</v>
       </c>
+      <c r="M6" s="13"/>
     </row>
     <row r="7" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D7" s="4">
+      <c r="D7" s="8">
         <v>74</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="9">
         <v>656789012</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="10">
         <v>35246</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="11" t="s">
-        <v>61</v>
-      </c>
+      <c r="M7" s="13"/>
     </row>
     <row r="8" spans="4:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="8">
@@ -825,9 +870,7 @@
       <c r="L8" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M8" s="12" t="s">
-        <v>62</v>
-      </c>
+      <c r="M8" s="13"/>
     </row>
     <row r="9" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D9" s="8">
@@ -947,11 +990,11 @@
       <c r="L12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="M12" s="13"/>
+      <c r="M12" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="M5:M12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Mise en place de la sécurité du site sur les URL, mise en en place d'un regex pour les mot de passe
</commit_message>
<xml_diff>
--- a/InfosUtilisateursSite.xlsx
+++ b/InfosUtilisateursSite.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemai\Documents\13_ProjetsPro\1_FormationDevWeb_2022_2023\Site_E-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B279E1FE-7C08-4B5B-824A-E84CBE95C6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A661400-BB12-42F7-AA3A-F6485E6B92E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="62">
   <si>
     <t>Nom</t>
   </si>
@@ -208,9 +208,6 @@
   </si>
   <si>
     <t>Tlemaire03022002.</t>
-  </si>
-  <si>
-    <t>USER Temporaire</t>
   </si>
   <si>
     <t xml:space="preserve">A rajouter
@@ -323,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -353,9 +350,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -719,31 +713,31 @@
       </c>
     </row>
     <row r="4" spans="4:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="4">
+      <c r="D4" s="8">
         <v>71</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="9">
         <v>623456789</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="10">
         <v>33810</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="9" t="s">
         <v>13</v>
       </c>
       <c r="M4" s="11" t="s">
@@ -778,9 +772,7 @@
       <c r="L5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="12" t="s">
-        <v>62</v>
-      </c>
+      <c r="M5" s="12"/>
     </row>
     <row r="6" spans="4:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D6" s="8">
@@ -810,7 +802,7 @@
       <c r="L6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M6" s="13"/>
+      <c r="M6" s="12"/>
     </row>
     <row r="7" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D7" s="8">
@@ -840,7 +832,7 @@
       <c r="L7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="13"/>
+      <c r="M7" s="12"/>
     </row>
     <row r="8" spans="4:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="8">
@@ -870,7 +862,7 @@
       <c r="L8" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M8" s="13"/>
+      <c r="M8" s="12"/>
     </row>
     <row r="9" spans="4:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D9" s="8">
@@ -900,7 +892,7 @@
       <c r="L9" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M9" s="13"/>
+      <c r="M9" s="12"/>
     </row>
     <row r="10" spans="4:13" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D10" s="8">
@@ -930,7 +922,7 @@
       <c r="L10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M10" s="13"/>
+      <c r="M10" s="12"/>
     </row>
     <row r="11" spans="4:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D11" s="8">
@@ -960,9 +952,9 @@
       <c r="L11" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M11" s="13"/>
-    </row>
-    <row r="12" spans="4:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M11" s="12"/>
+    </row>
+    <row r="12" spans="4:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D12" s="5">
         <v>79</v>
       </c>
@@ -990,11 +982,11 @@
       <c r="L12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="M12" s="14"/>
+      <c r="M12" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="M5:M12"/>
+    <mergeCell ref="M4:M12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
reorganisation du code, mise en place de commentaire si necessaire dans les fichiers, reglages de plusieurs details sur le site. Finalisation du site en V1
</commit_message>
<xml_diff>
--- a/InfosUtilisateursSite.xlsx
+++ b/InfosUtilisateursSite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lemai\Documents\13_ProjetsPro\1_FormationDevWeb_2022_2023\Site_E-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A661400-BB12-42F7-AA3A-F6485E6B92E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DCC030-127B-45A1-BD79-D6B5AD7A47E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="3045" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -78,9 +78,6 @@
     <t>claire.dupont@example.com</t>
   </si>
   <si>
-    <t>Pass!9A</t>
-  </si>
-  <si>
     <t>cdupont</t>
   </si>
   <si>
@@ -213,6 +210,9 @@
     <t xml:space="preserve">A rajouter
 Apres
 </t>
+  </si>
+  <si>
+    <t>Pass!9A.</t>
   </si>
 </sst>
 </file>
@@ -656,7 +656,7 @@
   <sheetData>
     <row r="2" spans="4:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>0</v>
@@ -726,10 +726,10 @@
         <v>16</v>
       </c>
       <c r="H4" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="9" t="s">
         <v>17</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>18</v>
       </c>
       <c r="J4" s="9">
         <v>623456789</v>
@@ -738,10 +738,7 @@
         <v>33810</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="4:13" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -749,19 +746,19 @@
         <v>72</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>23</v>
       </c>
       <c r="J5" s="9">
         <v>634567890</v>
@@ -772,26 +769,28 @@
       <c r="L5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="12"/>
+      <c r="M5" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="6" spans="4:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D6" s="8">
         <v>73</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>28</v>
       </c>
       <c r="J6" s="9">
         <v>645678901</v>
@@ -809,19 +808,19 @@
         <v>74</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>32</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>33</v>
       </c>
       <c r="J7" s="9">
         <v>656789012</v>
@@ -839,19 +838,19 @@
         <v>75</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="G8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="H8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>37</v>
       </c>
       <c r="J8" s="9">
         <v>667890123</v>
@@ -860,7 +859,7 @@
         <v>36783</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M8" s="12"/>
     </row>
@@ -869,19 +868,19 @@
         <v>76</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="J9" s="9">
         <v>678901234</v>
@@ -890,7 +889,7 @@
         <v>34670</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M9" s="12"/>
     </row>
@@ -899,19 +898,19 @@
         <v>77</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="H10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="I10" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>48</v>
       </c>
       <c r="J10" s="9">
         <v>689012345</v>
@@ -920,7 +919,7 @@
         <v>35541</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M10" s="12"/>
     </row>
@@ -929,19 +928,19 @@
         <v>78</v>
       </c>
       <c r="E11" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>53</v>
       </c>
       <c r="J11" s="9">
         <v>690123456</v>
@@ -950,7 +949,7 @@
         <v>33460</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M11" s="12"/>
     </row>
@@ -959,19 +958,19 @@
         <v>79</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="J12" s="6">
         <v>601234567</v>
@@ -980,13 +979,13 @@
         <v>36285</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M12" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="M4:M12"/>
+    <mergeCell ref="M5:M12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>